<commit_message>
Tasks.xlsx: certification test task 16 closed (ACT-0854f55fe0, Gev-approved, VERIFIED)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tasks.xlsx
+++ b/Tasks.xlsx
@@ -15,10 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -381,7 +380,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -637,7 +636,8 @@
     <xf numFmtId="164" fontId="14" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1881,15 +1881,15 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Չսկսված</t>
+          <t>Արված</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Mission 4.2 live certification · harmless · Gev-approved · cleanup = close/remove this row</t>
-        </is>
-      </c>
-      <c r="K28" s="107" t="n">
+          <t>Mission 4.2 live certification · harmless · Gev-approved · cleanup = close/remove this row · closed: live write certification completed: ACT-ef5fb6b5d0 VERIFIED by read-back (row 28, id 16)</t>
+        </is>
+      </c>
+      <c r="K28" s="108" t="n">
         <v>46277</v>
       </c>
       <c r="L28" t="inlineStr">
@@ -2353,8 +2353,8 @@
   <mergeCells count="74">
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="L15:N15"/>
+    <mergeCell ref="F5:H5"/>
     <mergeCell ref="L24:N24"/>
-    <mergeCell ref="F5:H5"/>
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="L18:N18"/>
     <mergeCell ref="L14:N14"/>

</xml_diff>